<commit_message>
changes in the presentation, running ui and videos
</commit_message>
<xml_diff>
--- a/data/pages.xlsx
+++ b/data/pages.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lioramitay/Documents/GitHub/Automation-Documentation/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D931D1B7-008D-294B-8C63-0EEAFDF0BA6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05DFCFF5-7087-4B44-B2CE-8F478B836B9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38400" yWindow="1140" windowWidth="38400" windowHeight="19200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38400" yWindow="600" windowWidth="38400" windowHeight="19200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Pages" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="77">
   <si>
     <t>file name</t>
   </si>
@@ -214,21 +214,6 @@
   </si>
   <si>
     <t>Part 9- Audit logs</t>
-  </si>
-  <si>
-    <t>Jeen Office Add-ins</t>
-  </si>
-  <si>
-    <t>Jeen for Excel — Product Spec</t>
-  </si>
-  <si>
-    <t>https://jeenai.atlassian.net/wiki/spaces/GKC/pages/443678721/Jeen+for+Excel+Product+Spec</t>
-  </si>
-  <si>
-    <t>Jeen for Outlook — Product Spec</t>
-  </si>
-  <si>
-    <t>https://jeenai.atlassian.net/wiki/spaces/GKC/pages/445906946/Jeen+for+Outlook+Product+Spec</t>
   </si>
   <si>
     <t>APIs &amp; Platform Interfaces</t>
@@ -645,7 +630,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C36"/>
+  <dimension ref="A1:C34"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="21.42578125" bestFit="1" customWidth="1"/>
@@ -779,7 +764,7 @@
         <v>25</v>
       </c>
       <c r="B12" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="C12" t="s">
         <v>26</v>
@@ -801,7 +786,7 @@
         <v>25</v>
       </c>
       <c r="B14" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="C14" t="s">
         <v>29</v>
@@ -886,24 +871,24 @@
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="B22" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="C22" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="B23" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="C23" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.2">
@@ -1007,46 +992,24 @@
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="B33" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="C33" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="B34" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="C34" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A35" t="s">
-        <v>64</v>
-      </c>
-      <c r="B35" t="s">
-        <v>65</v>
-      </c>
-      <c r="C35" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A36" t="s">
-        <v>64</v>
-      </c>
-      <c r="B36" t="s">
-        <v>67</v>
-      </c>
-      <c r="C36" t="s">
-        <v>68</v>
+        <v>76</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
changes in generation presentation and videos - 24/6
</commit_message>
<xml_diff>
--- a/data/pages.xlsx
+++ b/data/pages.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lioramitay/Documents/GitHub/Automation-Documentation/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05DFCFF5-7087-4B44-B2CE-8F478B836B9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A6F93CB-E0DC-1D48-ABF0-D3BFF846F11F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-38400" yWindow="600" windowWidth="38400" windowHeight="19200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="81">
   <si>
     <t>file name</t>
   </si>
@@ -228,12 +228,6 @@
     <t>Skills</t>
   </si>
   <si>
-    <t>Part 1 - Skills</t>
-  </si>
-  <si>
-    <t>https://jeenai.atlassian.net/wiki/spaces/GKC/pages/382468165/Part+1+-+Skills</t>
-  </si>
-  <si>
     <t>Part 1 - Uploading and Processing Documents</t>
   </si>
   <si>
@@ -254,6 +248,24 @@
   </si>
   <si>
     <t>https://jeenai.atlassian.net/wiki/spaces/GKC/pages/492666964/Part+2+-finOps+Wallets+System+and+Core+Capabilities</t>
+  </si>
+  <si>
+    <t>Part 1- Skills Fundamentals</t>
+  </si>
+  <si>
+    <t>https://jeenai.atlassian.net/wiki/spaces/GKC/pages/382468165/Part+1-+Skills+Fundamentals</t>
+  </si>
+  <si>
+    <t>Part 2 - Creating, Using and Managing Skills</t>
+  </si>
+  <si>
+    <t>https://jeenai.atlassian.net/wiki/spaces/GKC/pages/502005766/Part+2+-+Creating+Using+and+Managing+Skills</t>
+  </si>
+  <si>
+    <t>Part 3 - Skill Structure, Best Practices and FAQ</t>
+  </si>
+  <si>
+    <t>https://jeenai.atlassian.net/wiki/spaces/GKC/pages/502071300/Part+3+-+Skill+Structure+Best+Practices+and+FAQ</t>
   </si>
 </sst>
 </file>
@@ -630,7 +642,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C34"/>
+  <dimension ref="A1:C36"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="21.42578125" bestFit="1" customWidth="1"/>
@@ -764,7 +776,7 @@
         <v>25</v>
       </c>
       <c r="B12" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="C12" t="s">
         <v>26</v>
@@ -786,7 +798,7 @@
         <v>25</v>
       </c>
       <c r="B14" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C14" t="s">
         <v>29</v>
@@ -874,43 +886,43 @@
         <v>67</v>
       </c>
       <c r="B22" t="s">
-        <v>68</v>
+        <v>75</v>
       </c>
       <c r="C22" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="B23" t="s">
-        <v>65</v>
+        <v>77</v>
       </c>
       <c r="C23" t="s">
-        <v>66</v>
+        <v>78</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>45</v>
+        <v>67</v>
       </c>
       <c r="B24" t="s">
-        <v>47</v>
+        <v>79</v>
       </c>
       <c r="C24" t="s">
-        <v>46</v>
+        <v>80</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>45</v>
+        <v>64</v>
       </c>
       <c r="B25" t="s">
-        <v>48</v>
+        <v>65</v>
       </c>
       <c r="C25" t="s">
-        <v>49</v>
+        <v>66</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.2">
@@ -918,10 +930,10 @@
         <v>45</v>
       </c>
       <c r="B26" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="C26" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.2">
@@ -929,10 +941,10 @@
         <v>45</v>
       </c>
       <c r="B27" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="C27" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.2">
@@ -940,10 +952,10 @@
         <v>45</v>
       </c>
       <c r="B28" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="C28" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.2">
@@ -951,10 +963,10 @@
         <v>45</v>
       </c>
       <c r="B29" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="C29" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.2">
@@ -962,10 +974,10 @@
         <v>45</v>
       </c>
       <c r="B30" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="C30" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.2">
@@ -973,10 +985,10 @@
         <v>45</v>
       </c>
       <c r="B31" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="C31" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.2">
@@ -984,39 +996,60 @@
         <v>45</v>
       </c>
       <c r="B32" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="C32" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>72</v>
+        <v>45</v>
       </c>
       <c r="B33" t="s">
-        <v>73</v>
+        <v>60</v>
       </c>
       <c r="C33" t="s">
-        <v>74</v>
+        <v>61</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
+        <v>45</v>
+      </c>
+      <c r="B34" t="s">
+        <v>63</v>
+      </c>
+      <c r="C34" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A35" t="s">
+        <v>70</v>
+      </c>
+      <c r="B35" t="s">
+        <v>71</v>
+      </c>
+      <c r="C35" t="s">
         <v>72</v>
       </c>
-      <c r="B34" t="s">
-        <v>75</v>
-      </c>
-      <c r="C34" t="s">
-        <v>76</v>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A36" t="s">
+        <v>70</v>
+      </c>
+      <c r="B36" t="s">
+        <v>73</v>
+      </c>
+      <c r="C36" t="s">
+        <v>74</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="C23" r:id="rId1" xr:uid="{A348E66F-BB85-6D43-9EB5-53CC0DFCF0EB}"/>
-    <hyperlink ref="C22" r:id="rId2" xr:uid="{4491AA8D-19FA-CD4C-B6B3-FA2C23A1873D}"/>
-    <hyperlink ref="C12" r:id="rId3" xr:uid="{BEA06312-3DE9-334B-A403-B3AD4B112954}"/>
+    <hyperlink ref="C25" r:id="rId1" xr:uid="{A348E66F-BB85-6D43-9EB5-53CC0DFCF0EB}"/>
+    <hyperlink ref="C12" r:id="rId2" xr:uid="{BEA06312-3DE9-334B-A403-B3AD4B112954}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>

</xml_diff>